<commit_message>
Cap nhat du lieu - 11/05/2026 15:42
</commit_message>
<xml_diff>
--- a/Tổng hợp.xlsx
+++ b/Tổng hợp.xlsx
@@ -523,9 +523,9 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>- KC: 3/2025
-- HT: 6/2025
-- QT: 7/2025</t>
+          <t>- KC: 3/2026
+- HT: 6/2026
+- QT: 7/2026</t>
         </is>
       </c>
       <c r="G2" t="n">

</xml_diff>